<commit_message>
List the NBE fields the application does not have; map them into the sheets
</commit_message>
<xml_diff>
--- a/templates/nbe/nbe-match-kyc.xlsx
+++ b/templates/nbe/nbe-match-kyc.xlsx
@@ -1186,14 +1186,26 @@
           <t>{{address2}}</t>
         </is>
       </c>
-      <c r="H2" s="6"/>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>{{isOtherCity}}</t>
+        </is>
+      </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
           <t>{{city}}</t>
         </is>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>{{state}}</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>{{country}}</t>
+        </is>
+      </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>{{zip}}</t>
@@ -1204,7 +1216,11 @@
           <t>{{phone0}}</t>
         </is>
       </c>
-      <c r="N2" s="6"/>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>{{altPhone0}}</t>
+        </is>
+      </c>
       <c r="O2" s="6"/>
       <c r="P2" s="6"/>
       <c r="Q2" s="5" t="inlineStr">
@@ -1222,29 +1238,61 @@
           <t>{{ownerFirst}}</t>
         </is>
       </c>
-      <c r="T2" s="6"/>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerMiddle}}</t>
+        </is>
+      </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
           <t>{{ownerLast}}</t>
         </is>
       </c>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerAddress1}}</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerAddress2}}</t>
+        </is>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerIsOtherCity}}</t>
+        </is>
+      </c>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>{{city}}</t>
+          <t>{{ownerCity}}</t>
         </is>
       </c>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="6"/>
-      <c r="AB2" s="6"/>
+      <c r="Z2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerState}}</t>
+        </is>
+      </c>
+      <c r="AA2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerCountry}}</t>
+        </is>
+      </c>
+      <c r="AB2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerZip}}</t>
+        </is>
+      </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
           <t>{{phone0}}</t>
         </is>
       </c>
-      <c r="AD2" s="6"/>
+      <c r="AD2" s="6" t="inlineStr">
+        <is>
+          <t>{{ownerAltPhone0}}</t>
+        </is>
+      </c>
       <c r="AE2" s="8" t="inlineStr">
         <is>
           <t>{{email}}</t>

</xml_diff>